<commit_message>
update logic and output
</commit_message>
<xml_diff>
--- a/rules/CORE-000852/negative/01/data/unit-test-coreid-CG0330-negative.xlsx
+++ b/rules/CORE-000852/negative/01/data/unit-test-coreid-CG0330-negative.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10920"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian\core-contributor\rules\CORE-000852\negative\01\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/CORE-000852/negative/01/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B848F65-4212-448F-9DAA-966AF154808A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82D157FF-5971-4C42-9C13-BAA89141B28F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30330" yWindow="855" windowWidth="23265" windowHeight="14505" tabRatio="576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30340" yWindow="860" windowWidth="23260" windowHeight="14500" tabRatio="576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="30" r:id="rId1"/>
@@ -818,7 +818,7 @@
     <t>$column_order_from_dataset</t>
   </si>
   <si>
-    <t>$column_order_from_library</t>
+    <t>$library_with_dataset_only</t>
   </si>
 </sst>
 </file>
@@ -959,7 +959,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -990,13 +990,7 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1933,9 +1927,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D962C8A-AFA1-4EE3-9E57-8981969F2E6E}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -1943,7 +1937,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1959,14 +1953,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="36.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="3.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="36.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1974,7 +1968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1982,7 +1976,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1990,7 +1984,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1998,7 +1992,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -2017,12 +2011,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BDDED82-7289-408A-8597-CE1381ED9DDD}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="5" max="5" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="11" t="s">
         <v>249</v>
       </c>
@@ -2042,7 +2036,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2059,7 +2053,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2076,7 +2070,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2093,7 +2087,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2</v>
       </c>
@@ -2110,7 +2104,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>3</v>
       </c>
@@ -2127,7 +2121,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>3</v>
       </c>
@@ -2144,7 +2138,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>4</v>
       </c>
@@ -2161,7 +2155,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>4</v>
       </c>
@@ -2180,23 +2174,24 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:U8"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="21" width="20.7109375" style="2" customWidth="1"/>
-    <col min="22" max="16384" width="8.85546875" style="2"/>
+    <col min="1" max="21" width="20.6640625" style="2" customWidth="1"/>
+    <col min="22" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -2257,7 +2252,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>33</v>
       </c>
@@ -2322,7 +2317,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>53</v>
       </c>
@@ -2387,7 +2382,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>50</v>
       </c>
@@ -2452,7 +2447,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>55</v>
       </c>
@@ -2509,7 +2504,7 @@
       <c r="T5"/>
       <c r="U5"/>
     </row>
-    <row r="6" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>55</v>
       </c>
@@ -2560,7 +2555,7 @@
       </c>
       <c r="U6" s="5"/>
     </row>
-    <row r="7" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>55</v>
       </c>
@@ -2616,7 +2611,7 @@
       </c>
       <c r="U7" s="4"/>
     </row>
-    <row r="8" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>55</v>
       </c>
@@ -2680,13 +2675,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B41BDCC7-F382-49D0-BD18-4F06A3554CB3}">
   <dimension ref="A1:R18"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="18" width="20.7109375" style="2" customWidth="1"/>
-    <col min="19" max="16384" width="8.85546875" style="2"/>
+    <col min="1" max="18" width="20.6640625" style="2" customWidth="1"/>
+    <col min="19" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>14</v>
       </c>
@@ -2717,7 +2712,7 @@
       <c r="J1" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" s="2" t="s">
         <v>245</v>
       </c>
       <c r="L1" s="2" t="s">
@@ -2742,7 +2737,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>33</v>
       </c>
@@ -2798,7 +2793,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>53</v>
       </c>
@@ -2854,7 +2849,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>50</v>
       </c>
@@ -2910,7 +2905,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>55</v>
       </c>
@@ -2950,7 +2945,7 @@
       </c>
       <c r="R5" s="5"/>
     </row>
-    <row r="6" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>55</v>
       </c>
@@ -2996,7 +2991,7 @@
       </c>
       <c r="R6" s="5"/>
     </row>
-    <row r="7" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>55</v>
       </c>
@@ -3036,7 +3031,7 @@
       </c>
       <c r="R7" s="5"/>
     </row>
-    <row r="8" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>55</v>
       </c>
@@ -3080,7 +3075,7 @@
       <c r="Q8" s="5"/>
       <c r="R8" s="5"/>
     </row>
-    <row r="9" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>55</v>
       </c>
@@ -3122,7 +3117,7 @@
       <c r="Q9" s="5"/>
       <c r="R9" s="5"/>
     </row>
-    <row r="10" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>55</v>
       </c>
@@ -3162,7 +3157,7 @@
       </c>
       <c r="R10" s="5"/>
     </row>
-    <row r="11" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>55</v>
       </c>
@@ -3204,7 +3199,7 @@
       <c r="Q11" s="5"/>
       <c r="R11" s="5"/>
     </row>
-    <row r="12" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>55</v>
       </c>
@@ -3246,7 +3241,7 @@
       </c>
       <c r="R12" s="5"/>
     </row>
-    <row r="13" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>55</v>
       </c>
@@ -3288,7 +3283,7 @@
       </c>
       <c r="R13" s="5"/>
     </row>
-    <row r="14" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
         <v>55</v>
       </c>
@@ -3330,7 +3325,7 @@
       <c r="Q14" s="5"/>
       <c r="R14" s="5"/>
     </row>
-    <row r="15" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
         <v>55</v>
       </c>
@@ -3378,7 +3373,7 @@
       <c r="Q15" s="5"/>
       <c r="R15" s="5"/>
     </row>
-    <row r="16" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
         <v>55</v>
       </c>
@@ -3420,7 +3415,7 @@
       <c r="Q16" s="5"/>
       <c r="R16" s="5"/>
     </row>
-    <row r="17" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
         <v>55</v>
       </c>
@@ -3462,7 +3457,7 @@
       <c r="Q17" s="5"/>
       <c r="R17" s="5"/>
     </row>
-    <row r="18" spans="1:18" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
         <v>55</v>
       </c>
@@ -3516,13 +3511,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E928109-8D06-4717-9DE5-10A023DB72D3}">
   <dimension ref="A1:X9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="24" width="20.7109375" style="5" customWidth="1"/>
+    <col min="1" max="24" width="20.6640625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:24" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
         <v>158</v>
       </c>
       <c r="B1" s="5" t="s">
@@ -3595,7 +3590,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>177</v>
       </c>
@@ -3669,7 +3664,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>53</v>
       </c>
@@ -3743,7 +3738,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" s="5">
         <v>19</v>
       </c>
@@ -3817,7 +3812,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>191</v>
       </c>
@@ -3879,7 +3874,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>198</v>
       </c>
@@ -3947,7 +3942,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>201</v>
       </c>
@@ -4009,7 +4004,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>205</v>
       </c>
@@ -4074,7 +4069,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>214</v>
       </c>
@@ -4165,13 +4160,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F69B0C80-0D21-48CC-B786-5AC734E98D04}">
   <dimension ref="A1:S9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="18" width="20.7109375" style="5" customWidth="1"/>
-    <col min="19" max="19" width="20.7109375" style="6" customWidth="1"/>
+    <col min="1" max="18" width="20.6640625" style="5" customWidth="1"/>
+    <col min="19" max="19" width="20.6640625" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>14</v>
       </c>
@@ -4196,7 +4191,7 @@
       <c r="H1" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="5" t="s">
         <v>221</v>
       </c>
       <c r="J1" s="5" t="s">
@@ -4230,7 +4225,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>33</v>
       </c>
@@ -4289,7 +4284,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>53</v>
       </c>
@@ -4348,7 +4343,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" s="5">
         <v>12</v>
       </c>
@@ -4407,7 +4402,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>55</v>
       </c>
@@ -4458,7 +4453,7 @@
       </c>
       <c r="S5" s="5"/>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>55</v>
       </c>
@@ -4506,7 +4501,7 @@
       </c>
       <c r="S6" s="5"/>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>55</v>
       </c>
@@ -4551,7 +4546,7 @@
       </c>
       <c r="S7" s="5"/>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>55</v>
       </c>
@@ -4596,7 +4591,7 @@
       </c>
       <c r="S8" s="5"/>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>55</v>
       </c>
@@ -4671,15 +4666,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010090ADB40D834AE945B19FCDA4041AC0CB" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c09bae7b217a3930fedb3a6204001e96">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9dee18c2-6da5-44c1-913e-bf7f393fe0e8" xmlns:ns3="63ea592b-d684-45c7-8cdc-fad8f8e6bb41" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac018b55a0c98af8ca0cc741473a0b1c" ns2:_="" ns3:_="">
     <xsd:import namespace="9dee18c2-6da5-44c1-913e-bf7f393fe0e8"/>
@@ -4902,6 +4888,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{68D2B826-D4BB-4F95-9EB6-C2567A4D352D}">
   <ds:schemaRefs>
@@ -4913,14 +4908,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3BEB11F-0E5C-4B66-89CC-AB3651412BF0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA37260-A745-4F1A-87F7-7324275C4FF1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4937,4 +4924,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3BEB11F-0E5C-4B66-89CC-AB3651412BF0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>